<commit_message>
Add Unit 2 guides, rename files, remove placeholders
Update repository with new Unit 2 study and lab materials, correct file numbering, and remove empty placeholder files. Changes include: updated Administracion attendance spreadsheet; added Unit 2 study guides for IDS/IPS and VPNs (DOCX and PDF); renamed Unit 2 study/lab files to correct session numbers (e.g. S31 -> S3, S1 -> S3); and deleted several .gitkeep placeholder files from image and lab guide folders.
</commit_message>
<xml_diff>
--- a/Administracion/Lista_Asistencia_ASS_CRN236396.xlsx
+++ b/Administracion/Lista_Asistencia_ASS_CRN236396.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5ddf5fb2bc65e958/Documentos/GitHub/lc_arquitectura_de_sistemas_de_seguridad/Administracion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{702E06F4-7ABE-4278-9F4F-32BE2150E49A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F70B20E0-8ED9-4973-A91C-E751630F28CA}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="14_{545CCF96-C524-4C47-965E-B405D4770607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{945EE14A-5570-4BC8-9146-5CEF22AA44DA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="857" uniqueCount="149">
   <si>
     <t>LISTA DE ASISTENCIA — ARQUITECTURA DE SISTEMAS DE SEGURIDAD  |  Ciclo 2026-A  |  CRN 236396  |  Sección 401  |  Aula 101 Edif. 4L</t>
   </si>
@@ -729,10 +729,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -845,10 +845,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1146,70 +1142,70 @@
       <c r="E3" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="22"/>
-      <c r="H3" s="23" t="s">
+      <c r="G3" s="23"/>
+      <c r="H3" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="22" t="s">
+      <c r="I3" s="22"/>
+      <c r="J3" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="K3" s="22"/>
-      <c r="L3" s="23" t="s">
+      <c r="K3" s="23"/>
+      <c r="L3" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="M3" s="23"/>
-      <c r="N3" s="22" t="s">
+      <c r="M3" s="22"/>
+      <c r="N3" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="O3" s="22"/>
-      <c r="P3" s="23" t="s">
+      <c r="O3" s="23"/>
+      <c r="P3" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="Q3" s="23"/>
-      <c r="R3" s="22" t="s">
+      <c r="Q3" s="22"/>
+      <c r="R3" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="S3" s="22"/>
-      <c r="T3" s="23" t="s">
+      <c r="S3" s="23"/>
+      <c r="T3" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="U3" s="23"/>
-      <c r="V3" s="22" t="s">
+      <c r="U3" s="22"/>
+      <c r="V3" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="W3" s="22"/>
-      <c r="X3" s="23" t="s">
+      <c r="W3" s="23"/>
+      <c r="X3" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="Y3" s="23"/>
-      <c r="Z3" s="22" t="s">
+      <c r="Y3" s="22"/>
+      <c r="Z3" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="AA3" s="22"/>
-      <c r="AB3" s="23" t="s">
+      <c r="AA3" s="23"/>
+      <c r="AB3" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="AC3" s="23"/>
-      <c r="AD3" s="22" t="s">
+      <c r="AC3" s="22"/>
+      <c r="AD3" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="AE3" s="22"/>
-      <c r="AF3" s="23" t="s">
+      <c r="AE3" s="23"/>
+      <c r="AF3" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="AG3" s="23"/>
-      <c r="AH3" s="22" t="s">
+      <c r="AG3" s="22"/>
+      <c r="AH3" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="AI3" s="22"/>
-      <c r="AJ3" s="23" t="s">
+      <c r="AI3" s="23"/>
+      <c r="AJ3" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="AK3" s="23"/>
+      <c r="AK3" s="22"/>
       <c r="AL3" s="4" t="s">
         <v>22</v>
       </c>
@@ -1497,17 +1493,21 @@
       <c r="V6" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W6" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="X6" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y6" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z6" s="12"/>
-      <c r="AA6" s="12"/>
+      <c r="W6" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X6" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y6" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z6" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA6" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="AB6" s="12"/>
       <c r="AC6" s="12"/>
       <c r="AD6" s="12"/>
@@ -1520,7 +1520,7 @@
       <c r="AK6" s="12"/>
       <c r="AL6" s="13">
         <f t="shared" ref="AL6:AL32" si="0">COUNTIF(F6,"A")+COUNTIF(G6,"A")+COUNTIF(H6,"A")+COUNTIF(I6,"A")+COUNTIF(J6,"A")+COUNTIF(K6,"A")+COUNTIF(L6,"A")+COUNTIF(M6,"A")+COUNTIF(N6,"A")+COUNTIF(O6,"A")+COUNTIF(P6,"A")+COUNTIF(Q6,"A")+COUNTIF(R6,"A")+COUNTIF(S6,"A")+COUNTIF(T6,"A")+COUNTIF(U6,"A")+COUNTIF(V6,"A")+COUNTIF(W6,"A")+COUNTIF(X6,"A")+COUNTIF(Y6,"A")+COUNTIF(Z6,"A")+COUNTIF(AA6,"A")+COUNTIF(AB6,"A")+COUNTIF(AC6,"A")+COUNTIF(AD6,"A")+COUNTIF(AE6,"A")+COUNTIF(AF6,"A")+COUNTIF(AG6,"A")+COUNTIF(AH6,"A")+COUNTIF(AI6,"A")+COUNTIF(AJ6,"A")+COUNTIF(AK6,"A")</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM6" s="14">
         <f t="shared" ref="AM6:AM32" si="1">COUNTIF(F6,"F")+COUNTIF(G6,"F")+COUNTIF(H6,"F")+COUNTIF(I6,"F")+COUNTIF(J6,"F")+COUNTIF(K6,"F")+COUNTIF(L6,"F")+COUNTIF(M6,"F")+COUNTIF(N6,"F")+COUNTIF(O6,"F")+COUNTIF(P6,"F")+COUNTIF(Q6,"F")+COUNTIF(R6,"F")+COUNTIF(S6,"F")+COUNTIF(T6,"F")+COUNTIF(U6,"F")+COUNTIF(V6,"F")+COUNTIF(W6,"F")+COUNTIF(X6,"F")+COUNTIF(Y6,"F")+COUNTIF(Z6,"F")+COUNTIF(AA6,"F")+COUNTIF(AB6,"F")+COUNTIF(AC6,"F")+COUNTIF(AD6,"F")+COUNTIF(AE6,"F")+COUNTIF(AF6,"F")+COUNTIF(AG6,"F")+COUNTIF(AH6,"F")+COUNTIF(AI6,"F")+COUNTIF(AJ6,"F")+COUNTIF(AK6,"F")</f>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="AN6" s="15">
         <f t="shared" ref="AN6:AN32" si="2">IF(AL6=0,"",AL6/32)</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="7" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1597,16 +1597,20 @@
         <v>146</v>
       </c>
       <c r="W7" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="X7" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="X7" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="Y7" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z7" s="19"/>
-      <c r="AA7" s="19"/>
+        <v>146</v>
+      </c>
+      <c r="Z7" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA7" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="AB7" s="19"/>
       <c r="AC7" s="19"/>
       <c r="AD7" s="19"/>
@@ -1619,7 +1623,7 @@
       <c r="AK7" s="19"/>
       <c r="AL7" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM7" s="14">
         <f t="shared" si="1"/>
@@ -1627,7 +1631,7 @@
       </c>
       <c r="AN7" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="8" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1695,17 +1699,21 @@
       <c r="V8" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W8" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="X8" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y8" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z8" s="12"/>
-      <c r="AA8" s="12"/>
+      <c r="W8" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X8" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y8" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z8" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA8" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="AB8" s="12"/>
       <c r="AC8" s="12"/>
       <c r="AD8" s="12"/>
@@ -1718,7 +1726,7 @@
       <c r="AK8" s="12"/>
       <c r="AL8" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM8" s="14">
         <f t="shared" si="1"/>
@@ -1726,7 +1734,7 @@
       </c>
       <c r="AN8" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="9" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1795,16 +1803,20 @@
         <v>146</v>
       </c>
       <c r="W9" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="X9" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="X9" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="Y9" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z9" s="19"/>
-      <c r="AA9" s="19"/>
+        <v>146</v>
+      </c>
+      <c r="Z9" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA9" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="AB9" s="19"/>
       <c r="AC9" s="19"/>
       <c r="AD9" s="19"/>
@@ -1817,7 +1829,7 @@
       <c r="AK9" s="19"/>
       <c r="AL9" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM9" s="14">
         <f t="shared" si="1"/>
@@ -1825,7 +1837,7 @@
       </c>
       <c r="AN9" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="10" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1841,7 +1853,9 @@
       <c r="D10" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="E10" s="11"/>
+      <c r="E10" s="11">
+        <v>1</v>
+      </c>
       <c r="F10" s="19" t="s">
         <v>145</v>
       </c>
@@ -1893,17 +1907,21 @@
       <c r="V10" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W10" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="X10" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y10" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z10" s="12"/>
-      <c r="AA10" s="12"/>
+      <c r="W10" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X10" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y10" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z10" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA10" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="AB10" s="12"/>
       <c r="AC10" s="12"/>
       <c r="AD10" s="12"/>
@@ -1916,7 +1934,7 @@
       <c r="AK10" s="12"/>
       <c r="AL10" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM10" s="14">
         <f t="shared" si="1"/>
@@ -1924,7 +1942,7 @@
       </c>
       <c r="AN10" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="11" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1993,16 +2011,20 @@
         <v>146</v>
       </c>
       <c r="W11" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="X11" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="X11" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="Y11" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z11" s="19"/>
-      <c r="AA11" s="19"/>
+        <v>146</v>
+      </c>
+      <c r="Z11" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA11" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="AB11" s="19"/>
       <c r="AC11" s="19"/>
       <c r="AD11" s="19"/>
@@ -2015,7 +2037,7 @@
       <c r="AK11" s="19"/>
       <c r="AL11" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM11" s="14">
         <f t="shared" si="1"/>
@@ -2023,7 +2045,7 @@
       </c>
       <c r="AN11" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="12" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2093,17 +2115,21 @@
       <c r="V12" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W12" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="X12" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y12" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z12" s="12"/>
-      <c r="AA12" s="12"/>
+      <c r="W12" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X12" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y12" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z12" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA12" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="AB12" s="12"/>
       <c r="AC12" s="12"/>
       <c r="AD12" s="12"/>
@@ -2116,7 +2142,7 @@
       <c r="AK12" s="12"/>
       <c r="AL12" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM12" s="14">
         <f t="shared" si="1"/>
@@ -2124,7 +2150,7 @@
       </c>
       <c r="AN12" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="13" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2193,16 +2219,20 @@
         <v>146</v>
       </c>
       <c r="W13" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="X13" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="X13" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="Y13" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z13" s="19"/>
-      <c r="AA13" s="19"/>
+        <v>146</v>
+      </c>
+      <c r="Z13" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA13" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="AB13" s="19"/>
       <c r="AC13" s="19"/>
       <c r="AD13" s="19"/>
@@ -2215,7 +2245,7 @@
       <c r="AK13" s="19"/>
       <c r="AL13" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM13" s="14">
         <f t="shared" si="1"/>
@@ -2223,7 +2253,7 @@
       </c>
       <c r="AN13" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="14" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2291,17 +2321,21 @@
       <c r="V14" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W14" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="X14" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y14" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z14" s="12"/>
-      <c r="AA14" s="12"/>
+      <c r="W14" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X14" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y14" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z14" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA14" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="AB14" s="12"/>
       <c r="AC14" s="12"/>
       <c r="AD14" s="12"/>
@@ -2314,7 +2348,7 @@
       <c r="AK14" s="12"/>
       <c r="AL14" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM14" s="14">
         <f t="shared" si="1"/>
@@ -2322,7 +2356,7 @@
       </c>
       <c r="AN14" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="15" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2393,16 +2427,20 @@
         <v>146</v>
       </c>
       <c r="W15" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="X15" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="X15" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="Y15" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z15" s="19"/>
-      <c r="AA15" s="19"/>
+        <v>146</v>
+      </c>
+      <c r="Z15" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA15" s="19" t="s">
+        <v>147</v>
+      </c>
       <c r="AB15" s="19"/>
       <c r="AC15" s="19"/>
       <c r="AD15" s="19"/>
@@ -2415,15 +2453,15 @@
       <c r="AK15" s="19"/>
       <c r="AL15" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="AM15" s="14">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN15" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.53125</v>
       </c>
     </row>
     <row r="16" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2491,17 +2529,21 @@
       <c r="V16" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W16" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="X16" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y16" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z16" s="12"/>
-      <c r="AA16" s="12"/>
+      <c r="W16" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X16" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y16" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z16" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA16" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="AB16" s="12"/>
       <c r="AC16" s="12"/>
       <c r="AD16" s="12"/>
@@ -2514,7 +2556,7 @@
       <c r="AK16" s="12"/>
       <c r="AL16" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM16" s="14">
         <f t="shared" si="1"/>
@@ -2522,7 +2564,7 @@
       </c>
       <c r="AN16" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="17" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2591,16 +2633,20 @@
         <v>146</v>
       </c>
       <c r="W17" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="X17" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="X17" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="Y17" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z17" s="19"/>
-      <c r="AA17" s="19"/>
+        <v>146</v>
+      </c>
+      <c r="Z17" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA17" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="AB17" s="19"/>
       <c r="AC17" s="19"/>
       <c r="AD17" s="19"/>
@@ -2617,7 +2663,7 @@
       </c>
       <c r="AM17" s="14">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN17" s="15">
         <f t="shared" si="2"/>
@@ -2689,17 +2735,21 @@
       <c r="V18" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W18" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="X18" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y18" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z18" s="12"/>
-      <c r="AA18" s="12"/>
+      <c r="W18" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X18" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y18" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z18" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA18" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="AB18" s="12"/>
       <c r="AC18" s="12"/>
       <c r="AD18" s="12"/>
@@ -2712,7 +2762,7 @@
       <c r="AK18" s="12"/>
       <c r="AL18" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM18" s="14">
         <f t="shared" si="1"/>
@@ -2720,7 +2770,7 @@
       </c>
       <c r="AN18" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="19" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2791,16 +2841,20 @@
         <v>146</v>
       </c>
       <c r="W19" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="X19" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="X19" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="Y19" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z19" s="19"/>
-      <c r="AA19" s="19"/>
+        <v>146</v>
+      </c>
+      <c r="Z19" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA19" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="AB19" s="19"/>
       <c r="AC19" s="19"/>
       <c r="AD19" s="19"/>
@@ -2813,7 +2867,7 @@
       <c r="AK19" s="19"/>
       <c r="AL19" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM19" s="14">
         <f t="shared" si="1"/>
@@ -2821,7 +2875,7 @@
       </c>
       <c r="AN19" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="20" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2889,17 +2943,21 @@
       <c r="V20" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W20" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="X20" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y20" s="12" t="s">
+      <c r="W20" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X20" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y20" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z20" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA20" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="Z20" s="12"/>
-      <c r="AA20" s="12"/>
       <c r="AB20" s="12"/>
       <c r="AC20" s="12"/>
       <c r="AD20" s="12"/>
@@ -2912,7 +2970,7 @@
       <c r="AK20" s="12"/>
       <c r="AL20" s="13">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AM20" s="14">
         <f t="shared" si="1"/>
@@ -2920,7 +2978,7 @@
       </c>
       <c r="AN20" s="15">
         <f t="shared" si="2"/>
-        <v>0.5625</v>
+        <v>0.53125</v>
       </c>
     </row>
     <row r="21" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2989,16 +3047,20 @@
         <v>146</v>
       </c>
       <c r="W21" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="X21" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="X21" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="Y21" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="Z21" s="19"/>
-      <c r="AA21" s="19"/>
+        <v>146</v>
+      </c>
+      <c r="Z21" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA21" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="AB21" s="19"/>
       <c r="AC21" s="19"/>
       <c r="AD21" s="19"/>
@@ -3015,7 +3077,7 @@
       </c>
       <c r="AM21" s="14">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN21" s="15">
         <f t="shared" si="2"/>
@@ -3087,17 +3149,21 @@
       <c r="V22" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W22" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="X22" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y22" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z22" s="12"/>
-      <c r="AA22" s="12"/>
+      <c r="W22" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X22" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y22" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z22" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA22" s="12" t="s">
+        <v>147</v>
+      </c>
       <c r="AB22" s="12"/>
       <c r="AC22" s="12"/>
       <c r="AD22" s="12"/>
@@ -3110,15 +3176,15 @@
       <c r="AK22" s="12"/>
       <c r="AL22" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="AM22" s="14">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN22" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.53125</v>
       </c>
     </row>
     <row r="23" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3187,16 +3253,20 @@
         <v>146</v>
       </c>
       <c r="W23" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="X23" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="X23" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="Y23" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z23" s="19"/>
-      <c r="AA23" s="19"/>
+        <v>146</v>
+      </c>
+      <c r="Z23" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA23" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="AB23" s="19"/>
       <c r="AC23" s="19"/>
       <c r="AD23" s="19"/>
@@ -3209,7 +3279,7 @@
       <c r="AK23" s="19"/>
       <c r="AL23" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM23" s="14">
         <f t="shared" si="1"/>
@@ -3217,7 +3287,7 @@
       </c>
       <c r="AN23" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="24" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3285,17 +3355,21 @@
       <c r="V24" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W24" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="X24" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y24" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z24" s="12"/>
-      <c r="AA24" s="12"/>
+      <c r="W24" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X24" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y24" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z24" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA24" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="AB24" s="12"/>
       <c r="AC24" s="12"/>
       <c r="AD24" s="12"/>
@@ -3308,7 +3382,7 @@
       <c r="AK24" s="12"/>
       <c r="AL24" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM24" s="14">
         <f t="shared" si="1"/>
@@ -3316,7 +3390,7 @@
       </c>
       <c r="AN24" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="25" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3385,16 +3459,20 @@
         <v>146</v>
       </c>
       <c r="W25" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="X25" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="X25" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="Y25" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z25" s="19"/>
-      <c r="AA25" s="19"/>
+        <v>146</v>
+      </c>
+      <c r="Z25" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA25" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="AB25" s="19"/>
       <c r="AC25" s="19"/>
       <c r="AD25" s="19"/>
@@ -3407,7 +3485,7 @@
       <c r="AK25" s="19"/>
       <c r="AL25" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM25" s="14">
         <f t="shared" si="1"/>
@@ -3415,7 +3493,7 @@
       </c>
       <c r="AN25" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="26" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3483,17 +3561,21 @@
       <c r="V26" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W26" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="X26" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y26" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z26" s="12"/>
-      <c r="AA26" s="12"/>
+      <c r="W26" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X26" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y26" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z26" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA26" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="AB26" s="12"/>
       <c r="AC26" s="12"/>
       <c r="AD26" s="12"/>
@@ -3506,7 +3588,7 @@
       <c r="AK26" s="12"/>
       <c r="AL26" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM26" s="14">
         <f t="shared" si="1"/>
@@ -3514,7 +3596,7 @@
       </c>
       <c r="AN26" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="27" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3583,16 +3665,20 @@
         <v>146</v>
       </c>
       <c r="W27" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="X27" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="X27" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="Y27" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z27" s="19"/>
-      <c r="AA27" s="19"/>
+        <v>146</v>
+      </c>
+      <c r="Z27" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA27" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="AB27" s="19"/>
       <c r="AC27" s="19"/>
       <c r="AD27" s="19"/>
@@ -3605,7 +3691,7 @@
       <c r="AK27" s="19"/>
       <c r="AL27" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM27" s="14">
         <f t="shared" si="1"/>
@@ -3613,7 +3699,7 @@
       </c>
       <c r="AN27" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="28" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3681,17 +3767,21 @@
       <c r="V28" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W28" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="X28" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y28" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="Z28" s="12"/>
-      <c r="AA28" s="12"/>
+      <c r="W28" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X28" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y28" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z28" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA28" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="AB28" s="12"/>
       <c r="AC28" s="12"/>
       <c r="AD28" s="12"/>
@@ -3704,15 +3794,15 @@
       <c r="AK28" s="12"/>
       <c r="AL28" s="13">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AM28" s="14">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AN28" s="15">
         <f t="shared" si="2"/>
-        <v>0.53125</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="29" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3728,7 +3818,9 @@
       <c r="D29" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="E29" s="18"/>
+      <c r="E29" s="18">
+        <v>1</v>
+      </c>
       <c r="F29" s="19" t="s">
         <v>145</v>
       </c>
@@ -3781,16 +3873,20 @@
         <v>146</v>
       </c>
       <c r="W29" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="X29" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="X29" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="Y29" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z29" s="19"/>
-      <c r="AA29" s="19"/>
+        <v>146</v>
+      </c>
+      <c r="Z29" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA29" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="AB29" s="19"/>
       <c r="AC29" s="19"/>
       <c r="AD29" s="19"/>
@@ -3803,7 +3899,7 @@
       <c r="AK29" s="19"/>
       <c r="AL29" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM29" s="14">
         <f t="shared" si="1"/>
@@ -3811,7 +3907,7 @@
       </c>
       <c r="AN29" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="30" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3881,17 +3977,21 @@
       <c r="V30" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W30" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="X30" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y30" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z30" s="12"/>
-      <c r="AA30" s="12"/>
+      <c r="W30" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X30" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y30" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z30" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA30" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="AB30" s="12"/>
       <c r="AC30" s="12"/>
       <c r="AD30" s="12"/>
@@ -3904,7 +4004,7 @@
       <c r="AK30" s="12"/>
       <c r="AL30" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM30" s="14">
         <f t="shared" si="1"/>
@@ -3912,7 +4012,7 @@
       </c>
       <c r="AN30" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="31" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3983,16 +4083,20 @@
         <v>146</v>
       </c>
       <c r="W31" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="X31" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="X31" s="19" t="s">
+        <v>146</v>
       </c>
       <c r="Y31" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z31" s="19"/>
-      <c r="AA31" s="19"/>
+        <v>146</v>
+      </c>
+      <c r="Z31" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA31" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="AB31" s="19"/>
       <c r="AC31" s="19"/>
       <c r="AD31" s="19"/>
@@ -4005,7 +4109,7 @@
       <c r="AK31" s="19"/>
       <c r="AL31" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM31" s="14">
         <f t="shared" si="1"/>
@@ -4013,7 +4117,7 @@
       </c>
       <c r="AN31" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="32" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4083,17 +4187,21 @@
       <c r="V32" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="W32" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="X32" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Y32" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="Z32" s="12"/>
-      <c r="AA32" s="12"/>
+      <c r="W32" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="X32" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y32" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="Z32" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="AA32" s="12" t="s">
+        <v>145</v>
+      </c>
       <c r="AB32" s="12"/>
       <c r="AC32" s="12"/>
       <c r="AD32" s="12"/>
@@ -4106,7 +4214,7 @@
       <c r="AK32" s="12"/>
       <c r="AL32" s="13">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AM32" s="14">
         <f t="shared" si="1"/>
@@ -4114,7 +4222,7 @@
       </c>
       <c r="AN32" s="15">
         <f t="shared" si="2"/>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="33" spans="1:40" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4195,23 +4303,23 @@
       </c>
       <c r="W33" s="20">
         <f t="shared" si="3"/>
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="X33" s="20">
         <f t="shared" si="3"/>
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="Y33" s="20">
         <f t="shared" si="3"/>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="Z33" s="20">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="AA33" s="20">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AB33" s="20">
         <f t="shared" si="3"/>
@@ -4303,7 +4411,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="AJ3:AK3"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="A34:AN34"/>
     <mergeCell ref="A1:AN1"/>
@@ -4323,6 +4430,7 @@
     <mergeCell ref="AD3:AE3"/>
     <mergeCell ref="AF3:AG3"/>
     <mergeCell ref="AH3:AI3"/>
+    <mergeCell ref="AJ3:AK3"/>
   </mergeCells>
   <conditionalFormatting sqref="AN6:AN32">
     <cfRule type="expression" dxfId="1" priority="2">
@@ -4404,7 +4512,7 @@
       </c>
       <c r="E3" s="13">
         <f>Asistencia!AL6</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F3" s="14">
         <f>Asistencia!AM6</f>
@@ -4412,7 +4520,7 @@
       </c>
       <c r="G3" s="15">
         <f>Asistencia!AN6</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H3" s="9" t="str">
         <f>IF(Asistencia!AN6="","Sin datos",IF(Asistencia!AN6&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4434,7 +4542,7 @@
       </c>
       <c r="E4" s="13">
         <f>Asistencia!AL7</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F4" s="14">
         <f>Asistencia!AM7</f>
@@ -4442,7 +4550,7 @@
       </c>
       <c r="G4" s="15">
         <f>Asistencia!AN7</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H4" s="16" t="str">
         <f>IF(Asistencia!AN7="","Sin datos",IF(Asistencia!AN7&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4464,7 +4572,7 @@
       </c>
       <c r="E5" s="13">
         <f>Asistencia!AL8</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F5" s="14">
         <f>Asistencia!AM8</f>
@@ -4472,7 +4580,7 @@
       </c>
       <c r="G5" s="15">
         <f>Asistencia!AN8</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H5" s="9" t="str">
         <f>IF(Asistencia!AN8="","Sin datos",IF(Asistencia!AN8&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4494,7 +4602,7 @@
       </c>
       <c r="E6" s="13">
         <f>Asistencia!AL9</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F6" s="14">
         <f>Asistencia!AM9</f>
@@ -4502,7 +4610,7 @@
       </c>
       <c r="G6" s="15">
         <f>Asistencia!AN9</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H6" s="16" t="str">
         <f>IF(Asistencia!AN9="","Sin datos",IF(Asistencia!AN9&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4524,7 +4632,7 @@
       </c>
       <c r="E7" s="13">
         <f>Asistencia!AL10</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F7" s="14">
         <f>Asistencia!AM10</f>
@@ -4532,7 +4640,7 @@
       </c>
       <c r="G7" s="15">
         <f>Asistencia!AN10</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H7" s="9" t="str">
         <f>IF(Asistencia!AN10="","Sin datos",IF(Asistencia!AN10&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4554,7 +4662,7 @@
       </c>
       <c r="E8" s="13">
         <f>Asistencia!AL11</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F8" s="14">
         <f>Asistencia!AM11</f>
@@ -4562,7 +4670,7 @@
       </c>
       <c r="G8" s="15">
         <f>Asistencia!AN11</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H8" s="16" t="str">
         <f>IF(Asistencia!AN11="","Sin datos",IF(Asistencia!AN11&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4584,7 +4692,7 @@
       </c>
       <c r="E9" s="13">
         <f>Asistencia!AL12</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F9" s="14">
         <f>Asistencia!AM12</f>
@@ -4592,7 +4700,7 @@
       </c>
       <c r="G9" s="15">
         <f>Asistencia!AN12</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H9" s="9" t="str">
         <f>IF(Asistencia!AN12="","Sin datos",IF(Asistencia!AN12&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4614,7 +4722,7 @@
       </c>
       <c r="E10" s="13">
         <f>Asistencia!AL13</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F10" s="14">
         <f>Asistencia!AM13</f>
@@ -4622,7 +4730,7 @@
       </c>
       <c r="G10" s="15">
         <f>Asistencia!AN13</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H10" s="16" t="str">
         <f>IF(Asistencia!AN13="","Sin datos",IF(Asistencia!AN13&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4644,7 +4752,7 @@
       </c>
       <c r="E11" s="13">
         <f>Asistencia!AL14</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F11" s="14">
         <f>Asistencia!AM14</f>
@@ -4652,7 +4760,7 @@
       </c>
       <c r="G11" s="15">
         <f>Asistencia!AN14</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H11" s="9" t="str">
         <f>IF(Asistencia!AN14="","Sin datos",IF(Asistencia!AN14&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4674,15 +4782,15 @@
       </c>
       <c r="E12" s="13">
         <f>Asistencia!AL15</f>
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F12" s="14">
         <f>Asistencia!AM15</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="15">
         <f>Asistencia!AN15</f>
-        <v>0.59375</v>
+        <v>0.53125</v>
       </c>
       <c r="H12" s="16" t="str">
         <f>IF(Asistencia!AN15="","Sin datos",IF(Asistencia!AN15&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4704,7 +4812,7 @@
       </c>
       <c r="E13" s="13">
         <f>Asistencia!AL16</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F13" s="14">
         <f>Asistencia!AM16</f>
@@ -4712,7 +4820,7 @@
       </c>
       <c r="G13" s="15">
         <f>Asistencia!AN16</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H13" s="9" t="str">
         <f>IF(Asistencia!AN16="","Sin datos",IF(Asistencia!AN16&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4738,7 +4846,7 @@
       </c>
       <c r="F14" s="14">
         <f>Asistencia!AM17</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" s="15">
         <f>Asistencia!AN17</f>
@@ -4764,7 +4872,7 @@
       </c>
       <c r="E15" s="13">
         <f>Asistencia!AL18</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F15" s="14">
         <f>Asistencia!AM18</f>
@@ -4772,7 +4880,7 @@
       </c>
       <c r="G15" s="15">
         <f>Asistencia!AN18</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H15" s="9" t="str">
         <f>IF(Asistencia!AN18="","Sin datos",IF(Asistencia!AN18&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4794,7 +4902,7 @@
       </c>
       <c r="E16" s="13">
         <f>Asistencia!AL19</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F16" s="14">
         <f>Asistencia!AM19</f>
@@ -4802,7 +4910,7 @@
       </c>
       <c r="G16" s="15">
         <f>Asistencia!AN19</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H16" s="16" t="str">
         <f>IF(Asistencia!AN19="","Sin datos",IF(Asistencia!AN19&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4824,7 +4932,7 @@
       </c>
       <c r="E17" s="13">
         <f>Asistencia!AL20</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F17" s="14">
         <f>Asistencia!AM20</f>
@@ -4832,7 +4940,7 @@
       </c>
       <c r="G17" s="15">
         <f>Asistencia!AN20</f>
-        <v>0.5625</v>
+        <v>0.53125</v>
       </c>
       <c r="H17" s="9" t="str">
         <f>IF(Asistencia!AN20="","Sin datos",IF(Asistencia!AN20&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4858,7 +4966,7 @@
       </c>
       <c r="F18" s="14">
         <f>Asistencia!AM21</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" s="15">
         <f>Asistencia!AN21</f>
@@ -4884,15 +4992,15 @@
       </c>
       <c r="E19" s="13">
         <f>Asistencia!AL22</f>
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F19" s="14">
         <f>Asistencia!AM22</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" s="15">
         <f>Asistencia!AN22</f>
-        <v>0.59375</v>
+        <v>0.53125</v>
       </c>
       <c r="H19" s="9" t="str">
         <f>IF(Asistencia!AN22="","Sin datos",IF(Asistencia!AN22&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4914,7 +5022,7 @@
       </c>
       <c r="E20" s="13">
         <f>Asistencia!AL23</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F20" s="14">
         <f>Asistencia!AM23</f>
@@ -4922,7 +5030,7 @@
       </c>
       <c r="G20" s="15">
         <f>Asistencia!AN23</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H20" s="16" t="str">
         <f>IF(Asistencia!AN23="","Sin datos",IF(Asistencia!AN23&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4944,7 +5052,7 @@
       </c>
       <c r="E21" s="13">
         <f>Asistencia!AL24</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F21" s="14">
         <f>Asistencia!AM24</f>
@@ -4952,7 +5060,7 @@
       </c>
       <c r="G21" s="15">
         <f>Asistencia!AN24</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H21" s="9" t="str">
         <f>IF(Asistencia!AN24="","Sin datos",IF(Asistencia!AN24&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -4974,7 +5082,7 @@
       </c>
       <c r="E22" s="13">
         <f>Asistencia!AL25</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F22" s="14">
         <f>Asistencia!AM25</f>
@@ -4982,7 +5090,7 @@
       </c>
       <c r="G22" s="15">
         <f>Asistencia!AN25</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H22" s="16" t="str">
         <f>IF(Asistencia!AN25="","Sin datos",IF(Asistencia!AN25&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -5004,7 +5112,7 @@
       </c>
       <c r="E23" s="13">
         <f>Asistencia!AL26</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F23" s="14">
         <f>Asistencia!AM26</f>
@@ -5012,7 +5120,7 @@
       </c>
       <c r="G23" s="15">
         <f>Asistencia!AN26</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H23" s="9" t="str">
         <f>IF(Asistencia!AN26="","Sin datos",IF(Asistencia!AN26&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -5034,7 +5142,7 @@
       </c>
       <c r="E24" s="13">
         <f>Asistencia!AL27</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F24" s="14">
         <f>Asistencia!AM27</f>
@@ -5042,7 +5150,7 @@
       </c>
       <c r="G24" s="15">
         <f>Asistencia!AN27</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H24" s="16" t="str">
         <f>IF(Asistencia!AN27="","Sin datos",IF(Asistencia!AN27&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -5064,15 +5172,15 @@
       </c>
       <c r="E25" s="13">
         <f>Asistencia!AL28</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F25" s="14">
         <f>Asistencia!AM28</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G25" s="15">
         <f>Asistencia!AN28</f>
-        <v>0.53125</v>
+        <v>0.5625</v>
       </c>
       <c r="H25" s="9" t="str">
         <f>IF(Asistencia!AN28="","Sin datos",IF(Asistencia!AN28&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -5094,7 +5202,7 @@
       </c>
       <c r="E26" s="13">
         <f>Asistencia!AL29</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F26" s="14">
         <f>Asistencia!AM29</f>
@@ -5102,7 +5210,7 @@
       </c>
       <c r="G26" s="15">
         <f>Asistencia!AN29</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H26" s="16" t="str">
         <f>IF(Asistencia!AN29="","Sin datos",IF(Asistencia!AN29&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -5124,7 +5232,7 @@
       </c>
       <c r="E27" s="13">
         <f>Asistencia!AL30</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F27" s="14">
         <f>Asistencia!AM30</f>
@@ -5132,7 +5240,7 @@
       </c>
       <c r="G27" s="15">
         <f>Asistencia!AN30</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H27" s="9" t="str">
         <f>IF(Asistencia!AN30="","Sin datos",IF(Asistencia!AN30&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -5154,7 +5262,7 @@
       </c>
       <c r="E28" s="13">
         <f>Asistencia!AL31</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F28" s="14">
         <f>Asistencia!AM31</f>
@@ -5162,7 +5270,7 @@
       </c>
       <c r="G28" s="15">
         <f>Asistencia!AN31</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H28" s="16" t="str">
         <f>IF(Asistencia!AN31="","Sin datos",IF(Asistencia!AN31&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>
@@ -5184,7 +5292,7 @@
       </c>
       <c r="E29" s="13">
         <f>Asistencia!AL32</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F29" s="14">
         <f>Asistencia!AM32</f>
@@ -5192,7 +5300,7 @@
       </c>
       <c r="G29" s="15">
         <f>Asistencia!AN32</f>
-        <v>0.59375</v>
+        <v>0.5625</v>
       </c>
       <c r="H29" s="9" t="str">
         <f>IF(Asistencia!AN32="","Sin datos",IF(Asistencia!AN32&gt;=0.8,"✅ Regular","⚠️ En riesgo"))</f>

</xml_diff>